<commit_message>
Derivados regenerados (catalogo 40.136 series, frescura, calidad) y presupuesto de catalogo
El catalogo crece con Italia por provincia y Grecia; el presupuesto de /catalogo.html?q=trigo sube 5213->5260 KB de datos y 810->822 KB gzip.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WpevEvgxxTSUSU4BwGMDZh
</commit_message>
<xml_diff>
--- a/data/pack/eu/trigo_duro.xlsx
+++ b/data/pack/eu/trigo_duro.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fuente y licencia" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuente y licencia" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,7 +502,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -557,7 +557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5617,7 +5617,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6607,7 +6607,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6772,7 +6772,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -7047,7 +7047,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7762,7 +7762,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -8257,7 +8257,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8312,7 +8312,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8477,7 +8477,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -8917,7 +8917,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -8972,7 +8972,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -9137,7 +9137,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -9192,7 +9192,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -9797,7 +9797,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -9852,7 +9852,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -10017,7 +10017,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -10072,7 +10072,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -10127,7 +10127,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -10237,7 +10237,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -10292,7 +10292,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -10457,7 +10457,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -10567,7 +10567,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -10787,7 +10787,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -10897,7 +10897,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -10952,7 +10952,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -11117,7 +11117,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -11392,7 +11392,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -11502,7 +11502,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -11557,7 +11557,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -11612,7 +11612,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -12162,7 +12162,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -12217,7 +12217,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -12327,7 +12327,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -12657,7 +12657,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -12712,7 +12712,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -12932,7 +12932,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -13042,7 +13042,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -13097,7 +13097,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -13152,7 +13152,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -13207,7 +13207,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -13262,7 +13262,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -13317,7 +13317,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -13427,7 +13427,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -13537,7 +13537,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -13757,7 +13757,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -13922,7 +13922,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -13977,7 +13977,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -14087,7 +14087,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -14142,7 +14142,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -14252,7 +14252,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -14417,7 +14417,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -14472,7 +14472,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -14637,7 +14637,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -14692,7 +14692,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -14747,7 +14747,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -14802,7 +14802,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -14857,7 +14857,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -14967,7 +14967,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -15187,7 +15187,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -15352,7 +15352,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -15407,7 +15407,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -15517,7 +15517,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -15682,7 +15682,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -15737,7 +15737,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -15847,7 +15847,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -15902,7 +15902,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -15957,7 +15957,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -16012,7 +16012,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -16122,7 +16122,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -16177,7 +16177,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -16232,7 +16232,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -16342,7 +16342,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -16452,7 +16452,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -16562,7 +16562,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -16617,7 +16617,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -16672,7 +16672,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -16727,7 +16727,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -16782,7 +16782,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -16892,7 +16892,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -17002,7 +17002,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -17057,7 +17057,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -17112,7 +17112,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -17167,7 +17167,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -17277,7 +17277,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -17387,7 +17387,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -17442,7 +17442,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -17497,7 +17497,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -17662,7 +17662,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -17717,7 +17717,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -17827,7 +17827,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -17937,7 +17937,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -17992,7 +17992,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -18047,7 +18047,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -18157,7 +18157,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -18212,7 +18212,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18322,7 +18322,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -18377,7 +18377,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -18432,7 +18432,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -18487,7 +18487,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -18542,7 +18542,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18597,7 +18597,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -18652,7 +18652,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -18707,7 +18707,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -18817,7 +18817,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -18872,7 +18872,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -18927,7 +18927,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -18982,7 +18982,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -19037,7 +19037,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -19092,7 +19092,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -19147,7 +19147,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -19202,7 +19202,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19257,7 +19257,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -19367,7 +19367,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -19422,7 +19422,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -19477,7 +19477,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -19587,7 +19587,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -19642,7 +19642,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19697,7 +19697,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -19752,7 +19752,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -19807,7 +19807,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19862,7 +19862,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19972,7 +19972,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -20027,7 +20027,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -20082,7 +20082,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -20137,7 +20137,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -20192,7 +20192,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -20247,7 +20247,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -20302,7 +20302,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20357,7 +20357,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20412,7 +20412,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -20467,7 +20467,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -20522,7 +20522,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -20577,7 +20577,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -20632,7 +20632,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20687,7 +20687,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20797,7 +20797,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20852,7 +20852,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20907,7 +20907,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -20962,7 +20962,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -21017,7 +21017,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -21127,7 +21127,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -21182,7 +21182,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -21237,7 +21237,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -21292,7 +21292,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -21347,7 +21347,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -21402,7 +21402,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -21457,7 +21457,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -21512,7 +21512,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -21677,7 +21677,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -21732,7 +21732,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -21787,7 +21787,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -21842,7 +21842,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -22007,7 +22007,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -22062,7 +22062,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -22117,7 +22117,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -22172,7 +22172,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -22227,7 +22227,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -22282,7 +22282,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -22337,7 +22337,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -22392,7 +22392,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -22447,7 +22447,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -22502,7 +22502,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -22557,7 +22557,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -22612,7 +22612,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -22667,7 +22667,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -22722,7 +22722,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -22777,7 +22777,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -22832,7 +22832,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -22887,7 +22887,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -22942,7 +22942,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -22997,7 +22997,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -23162,7 +23162,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -23217,7 +23217,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -23272,7 +23272,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -23327,7 +23327,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -23382,7 +23382,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -23492,7 +23492,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -23602,7 +23602,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -23657,7 +23657,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -23712,7 +23712,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -23767,7 +23767,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -23822,7 +23822,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -23877,7 +23877,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -23932,7 +23932,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -23987,7 +23987,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -24042,7 +24042,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -24097,7 +24097,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -24152,7 +24152,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>trigo_duro</t>
+          <t>Trigo duro</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -24225,7 +24225,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>trigo_duro (trigo_duro)</t>
+          <t>Trigo duro (trigo_duro)</t>
         </is>
       </c>
     </row>
@@ -24237,7 +24237,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>EU · Sevilla (España)</t>
         </is>
       </c>
     </row>
@@ -24247,7 +24247,11 @@
           <t>Descripcion del dato</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Comisión Europea, Agri-food Data Portal: precio semanal del trigo duro en el mercado de Sevilla (España), salida de silo tras almacenamiento en camión, EUR/tonelada. Es un mercado regional, no la media nacional (la media nacional del portal está desactualizada) ni un futuro. Italia, el mayor productor de la UE, publica sus propios mercados (Bolonia, Roma, Foggia…): se ven al elegir Italia y en la página de Europa. La API no publica fecha de publicación: se registra el día en que se recuperó por primera vez.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">

</xml_diff>